<commit_message>
Updated NZL_grids model - 2025-09-19 01:01
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_NZL_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA438199-708E-4F07-BC4D-82ADA6D37F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82188418-9902-42D3-8EBC-145AE3158EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -844,24 +844,96 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_015</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_002</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 2</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_006</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 6</t>
   </si>
   <si>
+    <t>distr_solelc_spv_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_013</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_007</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_012</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 12</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_010</t>
   </si>
   <si>
@@ -874,130 +946,106 @@
     <t>connecting solar to buses in cluster 3</t>
   </si>
   <si>
-    <t>distr_solelc_spv_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_007</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_012</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_013</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_015</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_w93419960-220,e_w409049317-220,e_w95512216-220,e_w270556206-220,e_w148300699-220,e_NZ13-220,e_w167283894-220</t>
+  </si>
+  <si>
+    <t>e_w180519027-220,e_w89636510-220,e_NZ30-220</t>
+  </si>
+  <si>
+    <t>e_w95046918-220,e_w95048289-220,e_NZ27-220,e_w167705537-220</t>
+  </si>
+  <si>
+    <t>e_w95046918-220,e_NZ27-220,e_w167705537-220,e_w95343089-220,e_w93713118-220,e_NZ26-220,e_w95344674-220,e_w1026587442-220</t>
+  </si>
+  <si>
     <t>e_w89943957-220,e_w232382576-220</t>
   </si>
   <si>
     <t>e_r17609399-220,e_w95344674-220,e_w191346761-220,e_w167572576-220,e_NZ23-220,e_NZ21-220</t>
   </si>
   <si>
+    <t>e_NZ31-220,e_NZ30-220,e_w1099619174-220,e_w95048289-220</t>
+  </si>
+  <si>
+    <t>e_w412588974-220,e_NZ41-220,e_w268841395-220,e_w180519027-220,e_NZ42-220</t>
+  </si>
+  <si>
+    <t>e_w167427251-220,e_w94053861-220,e_w89411122-220,e_NZ14-220</t>
+  </si>
+  <si>
+    <t>e_w89637277-220,e_w94840399-220,e_NZ32-220,e_w167286837-220,e_w268826084-220</t>
+  </si>
+  <si>
+    <t>e_w268841395-220,e_w90092620-220,e_w180514007-220,e_w270521928-220</t>
+  </si>
+  <si>
+    <t>e_w412589726-220,e_w180519027-220</t>
+  </si>
+  <si>
+    <t>e_NZ40-220,e_w180519027-220,e_w414953388-220,e_NZ38-220,e_w89636510-220</t>
+  </si>
+  <si>
+    <t>e_w1099619174-220,e_w93827784-220,e_w100957314-220,e_w95046918-220</t>
+  </si>
+  <si>
     <t>e_NZ41-220</t>
   </si>
   <si>
     <t>e_w26671244-220,e_w61853727-220,e_w167293888-220,e_NZ3-220,e_w82881422-220,e_w270022030-220,e_w119877500-220,e_NZ5-220</t>
   </si>
   <si>
-    <t>e_NZ31-220,e_NZ30-220,e_w1099619174-220,e_w95048289-220</t>
-  </si>
-  <si>
-    <t>e_w412589726-220,e_w180519027-220</t>
-  </si>
-  <si>
-    <t>e_NZ40-220,e_w180519027-220,e_w414953388-220,e_NZ38-220,e_w89636510-220</t>
-  </si>
-  <si>
-    <t>e_w1099619174-220,e_w93827784-220,e_w100957314-220,e_w95046918-220</t>
-  </si>
-  <si>
-    <t>e_w89637277-220,e_w94840399-220,e_NZ32-220,e_w167286837-220,e_w268826084-220</t>
-  </si>
-  <si>
-    <t>e_w93419960-220,e_w409049317-220,e_w95512216-220,e_w270556206-220,e_w148300699-220,e_NZ13-220,e_w167283894-220</t>
-  </si>
-  <si>
-    <t>e_w167427251-220,e_w94053861-220,e_w89411122-220,e_NZ14-220</t>
-  </si>
-  <si>
-    <t>e_w268841395-220,e_w90092620-220,e_w180514007-220,e_w270521928-220</t>
-  </si>
-  <si>
-    <t>e_w180519027-220,e_w89636510-220,e_NZ30-220</t>
-  </si>
-  <si>
-    <t>e_w95046918-220,e_w95048289-220,e_NZ27-220,e_w167705537-220</t>
-  </si>
-  <si>
-    <t>e_w95046918-220,e_NZ27-220,e_w167705537-220,e_w95343089-220,e_w93713118-220,e_NZ26-220,e_w95344674-220,e_w1026587442-220</t>
-  </si>
-  <si>
-    <t>e_w412588974-220,e_NZ41-220,e_w268841395-220,e_w180519027-220,e_NZ42-220</t>
+    <t>distr_wonelc_won_015</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_002</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_008</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_011</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_012</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 12</t>
   </si>
   <si>
     <t>distr_wonelc_won_009</t>
@@ -1006,6 +1054,24 @@
     <t>connecting wind onshore to buses in cluster 9</t>
   </si>
   <si>
+    <t>distr_wonelc_won_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_007</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_014</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 14</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_005</t>
   </si>
   <si>
@@ -1024,70 +1090,52 @@
     <t>connecting wind onshore to buses in cluster 13</t>
   </si>
   <si>
-    <t>distr_wonelc_won_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_007</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_008</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_002</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_014</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_011</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_012</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_015</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
+    <t>elc_won_015</t>
+  </si>
+  <si>
+    <t>e_w95048289-220,e_NZ27-220</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>e_w89943957-220,e_w232382576-220,e_w26671244-220,e_w61853727-220,e_w167293888-220,e_NZ3-220,e_w82881422-220,e_w119877500-220,e_NZ5-220</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>e_w95048289-220,e_w167705537-220,e_r17609399-220,e_NZ26-220,e_w95344674-220,e_w191346761-220,e_w1026587442-220,e_w167572576-220,e_NZ23-220,e_NZ21-220</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>e_w167705537-220,e_w95343089-220,e_w93713118-220,e_w1026587442-220</t>
+  </si>
+  <si>
+    <t>elc_won_008</t>
+  </si>
+  <si>
+    <t>e_NZ41-220,e_w412589726-220,e_w268841395-220,e_w180519027-220</t>
+  </si>
+  <si>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>e_NZ41-220,e_w412589726-220,e_w180519027-220,e_w89636510-220</t>
+  </si>
+  <si>
+    <t>elc_won_011</t>
+  </si>
+  <si>
+    <t>e_w167286837-220,e_w268826084-220,e_w1099619174-220,e_w100957314-220,e_w93827784-220</t>
+  </si>
+  <si>
+    <t>elc_won_012</t>
+  </si>
+  <si>
+    <t>e_w95048289-220,e_w95046918-220,e_NZ27-220</t>
   </si>
   <si>
     <t>elc_won_009</t>
@@ -1096,6 +1144,24 @@
     <t>e_NZ41-220,e_w412588974-220,e_w268841395-220,e_NZ42-220</t>
   </si>
   <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>e_w167427251-220,e_w94053861-220,e_w89411122-220,e_NZ14-220,e_w270022030-220</t>
+  </si>
+  <si>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>e_w90092620-220,e_w180514007-220,e_w270521928-220,e_w89637277-220,e_w94840399-220</t>
+  </si>
+  <si>
+    <t>elc_won_014</t>
+  </si>
+  <si>
+    <t>e_NZ30-220,e_w1099619174-220</t>
+  </si>
+  <si>
     <t>elc_won_005</t>
   </si>
   <si>
@@ -1111,70 +1177,130 @@
     <t>e_NZ31-220,e_w268826084-220,e_w1099619174-220,e_w93827784-220,e_w95046918-220</t>
   </si>
   <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>e_w167705537-220,e_w95343089-220,e_w93713118-220,e_w1026587442-220</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>e_w90092620-220,e_w180514007-220,e_w270521928-220,e_w89637277-220,e_w94840399-220</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>e_NZ41-220,e_w412589726-220,e_w268841395-220,e_w180519027-220</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>e_w95048289-220,e_w167705537-220,e_r17609399-220,e_NZ26-220,e_w95344674-220,e_w191346761-220,e_w1026587442-220,e_w167572576-220,e_NZ23-220,e_NZ21-220</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>e_NZ30-220,e_w1099619174-220</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>e_w89943957-220,e_w232382576-220,e_w26671244-220,e_w61853727-220,e_w167293888-220,e_NZ3-220,e_w82881422-220,e_w119877500-220,e_NZ5-220</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>e_NZ41-220,e_w412589726-220,e_w180519027-220,e_w89636510-220</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>e_w167286837-220,e_w268826084-220,e_w1099619174-220,e_w100957314-220,e_w93827784-220</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>e_w95048289-220,e_w95046918-220,e_NZ27-220</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>e_w95048289-220,e_NZ27-220</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>e_w167427251-220,e_w94053861-220,e_w89411122-220,e_NZ14-220,e_w270022030-220</t>
+    <t>distr_wofelc_wof_019</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_027</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 27</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_020</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 20</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_003</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_008</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_016</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_009</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_025</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 25</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_023</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 23</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_029</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 29</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_015</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_021</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 21</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_031</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 31</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_030</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 30</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_014</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_028</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 28</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_033</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 33</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_002</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_010</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_007</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_017</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 17</t>
   </si>
   <si>
     <t>distr_wofelc_wof_026</t>
@@ -1183,36 +1309,6 @@
     <t>connecting wind offshore to buses in cluster 26</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_015</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_020</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 20</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_003</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_008</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_029</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 29</t>
-  </si>
-  <si>
     <t>distr_wofelc_wof_018</t>
   </si>
   <si>
@@ -1225,52 +1321,16 @@
     <t>connecting wind offshore to buses in cluster 5</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_016</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_009</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_025</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 25</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_023</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 23</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_010</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_007</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_017</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_021</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 21</t>
+    <t>distr_wofelc_wof_022</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 22</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
   </si>
   <si>
     <t>distr_wofelc_wof_024</t>
@@ -1297,36 +1357,6 @@
     <t>connecting wind offshore to buses in cluster 1</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_031</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 31</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_014</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_028</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 28</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_033</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 33</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_002</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 2</t>
-  </si>
-  <si>
     <t>distr_wofelc_wof_013</t>
   </si>
   <si>
@@ -1345,34 +1375,121 @@
     <t>connecting wind offshore to buses in cluster 4</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_022</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 22</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_019</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_027</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 27</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_030</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 30</t>
+    <t>elc_wof_019</t>
+  </si>
+  <si>
+    <t>e_w412588974-220,e_NZ42-220,e_w270521928-220</t>
+  </si>
+  <si>
+    <t>elc_wof_027</t>
+  </si>
+  <si>
+    <t>e_NZ30-220,e_w95048289-220</t>
+  </si>
+  <si>
+    <t>elc_wof_020</t>
+  </si>
+  <si>
+    <t>e_w412589726-220</t>
+  </si>
+  <si>
+    <t>elc_wof_003</t>
+  </si>
+  <si>
+    <t>elc_wof_008</t>
+  </si>
+  <si>
+    <t>e_w188180344-220,e_w61853727-220</t>
+  </si>
+  <si>
+    <t>elc_wof_016</t>
+  </si>
+  <si>
+    <t>e_NZ41-220,e_w412588974-220,e_w270521928-220</t>
+  </si>
+  <si>
+    <t>elc_wof_009</t>
+  </si>
+  <si>
+    <t>e_r17609399-220</t>
+  </si>
+  <si>
+    <t>elc_wof_025</t>
+  </si>
+  <si>
+    <t>e_w100957314-220,e_w93827784-220,e_w95046918-220</t>
+  </si>
+  <si>
+    <t>elc_wof_023</t>
+  </si>
+  <si>
+    <t>e_w100957314-220,e_w95343089-220,e_w93713118-220,e_w1026587442-220</t>
+  </si>
+  <si>
+    <t>elc_wof_029</t>
+  </si>
+  <si>
+    <t>elc_wof_015</t>
+  </si>
+  <si>
+    <t>e_w412588974-220</t>
+  </si>
+  <si>
+    <t>elc_wof_021</t>
+  </si>
+  <si>
+    <t>e_NZ41-220,e_w412589726-220,e_w412588974-220</t>
+  </si>
+  <si>
+    <t>elc_wof_031</t>
+  </si>
+  <si>
+    <t>e_w93713118-220,e_w1167708390-220,e_w1026587442-220,e_w167572576-220,e_w93419960-220</t>
+  </si>
+  <si>
+    <t>elc_wof_030</t>
+  </si>
+  <si>
+    <t>e_w95048289-220,e_NZ27-220,e_r17609399-220,e_w167705537-220</t>
+  </si>
+  <si>
+    <t>elc_wof_014</t>
+  </si>
+  <si>
+    <t>e_w412588974-220,e_NZ41-220</t>
+  </si>
+  <si>
+    <t>elc_wof_028</t>
+  </si>
+  <si>
+    <t>elc_wof_033</t>
+  </si>
+  <si>
+    <t>e_w95046918-220,e_w95343089-220,e_w93713118-220</t>
+  </si>
+  <si>
+    <t>elc_wof_002</t>
+  </si>
+  <si>
+    <t>e_w89943957-220</t>
+  </si>
+  <si>
+    <t>elc_wof_010</t>
+  </si>
+  <si>
+    <t>e_w232382576-220,e_w89943957-220,e_w1363994055-220,e_w82881422-220,e_NZ3-220</t>
+  </si>
+  <si>
+    <t>elc_wof_007</t>
+  </si>
+  <si>
+    <t>e_w167427251-220,e_NZ9-220,e_w167293888-220,e_NZ8-220,e_NZ5-220</t>
+  </si>
+  <si>
+    <t>elc_wof_017</t>
+  </si>
+  <si>
+    <t>e_w89637277-220,e_w100957314-220,e_w93713118-220</t>
   </si>
   <si>
     <t>elc_wof_026</t>
@@ -1381,33 +1498,6 @@
     <t>e_w167286837-220,e_w268826084-220,e_NZ29-220,e_w100957314-220</t>
   </si>
   <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>e_w412588974-220</t>
-  </si>
-  <si>
-    <t>elc_wof_020</t>
-  </si>
-  <si>
-    <t>e_w412589726-220</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>e_w188180344-220,e_w61853727-220</t>
-  </si>
-  <si>
-    <t>elc_wof_029</t>
-  </si>
-  <si>
-    <t>e_NZ30-220,e_w95048289-220</t>
-  </si>
-  <si>
     <t>elc_wof_018</t>
   </si>
   <si>
@@ -1420,52 +1510,16 @@
     <t>e_w95512216-220,e_NZ13-220</t>
   </si>
   <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>e_NZ41-220,e_w412588974-220,e_w270521928-220</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>e_r17609399-220</t>
-  </si>
-  <si>
-    <t>elc_wof_025</t>
-  </si>
-  <si>
-    <t>e_w100957314-220,e_w93827784-220,e_w95046918-220</t>
-  </si>
-  <si>
-    <t>elc_wof_023</t>
-  </si>
-  <si>
-    <t>e_w100957314-220,e_w95343089-220,e_w93713118-220,e_w1026587442-220</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>e_w232382576-220,e_w89943957-220,e_w1363994055-220,e_w82881422-220,e_NZ3-220</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>e_w167427251-220,e_NZ9-220,e_w167293888-220,e_NZ8-220,e_NZ5-220</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>e_w89637277-220,e_w100957314-220,e_w93713118-220</t>
-  </si>
-  <si>
-    <t>elc_wof_021</t>
-  </si>
-  <si>
-    <t>e_NZ41-220,e_w412589726-220,e_w412588974-220</t>
+    <t>elc_wof_022</t>
+  </si>
+  <si>
+    <t>e_w100957314-220,e_w95343089-220</t>
+  </si>
+  <si>
+    <t>elc_wof_006</t>
+  </si>
+  <si>
+    <t>e_w93419960-220,e_w95512216-220</t>
   </si>
   <si>
     <t>elc_wof_024</t>
@@ -1489,33 +1543,6 @@
     <t>elc_wof_001</t>
   </si>
   <si>
-    <t>e_w89943957-220</t>
-  </si>
-  <si>
-    <t>elc_wof_031</t>
-  </si>
-  <si>
-    <t>e_w93713118-220,e_w1167708390-220,e_w1026587442-220,e_w167572576-220,e_w93419960-220</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>e_w412588974-220,e_NZ41-220</t>
-  </si>
-  <si>
-    <t>elc_wof_028</t>
-  </si>
-  <si>
-    <t>elc_wof_033</t>
-  </si>
-  <si>
-    <t>e_w95046918-220,e_w95343089-220,e_w93713118-220</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
     <t>elc_wof_013</t>
   </si>
   <si>
@@ -1532,33 +1559,6 @@
   </si>
   <si>
     <t>e_w95512216-220,e_NZ13-220,e_w167283894-220</t>
-  </si>
-  <si>
-    <t>elc_wof_022</t>
-  </si>
-  <si>
-    <t>e_w100957314-220,e_w95343089-220</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>e_w93419960-220,e_w95512216-220</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
-  </si>
-  <si>
-    <t>e_w412588974-220,e_NZ42-220,e_w270521928-220</t>
-  </si>
-  <si>
-    <t>elc_wof_027</t>
-  </si>
-  <si>
-    <t>elc_wof_030</t>
-  </si>
-  <si>
-    <t>e_w95048289-220,e_NZ27-220,e_r17609399-220,e_w167705537-220</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -6777,7 +6777,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3F7E0EE-A8C0-4D08-90A3-D373DDDDB3E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27C11669-6791-4422-8D49-365020E06D77}">
   <dimension ref="B9:BD43"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7015,16 +7015,16 @@
         <v>238</v>
       </c>
       <c r="Y11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Z11" t="s">
         <v>274</v>
       </c>
       <c r="AA11">
-        <v>0.99541580702824473</v>
+        <v>0.99649838493007836</v>
       </c>
       <c r="AB11">
-        <v>84.0435378155141</v>
+        <v>64.196276281897482</v>
       </c>
       <c r="AD11" t="s">
         <v>237</v>
@@ -7057,10 +7057,10 @@
         <v>321</v>
       </c>
       <c r="AO11">
-        <v>0.9975157188831717</v>
+        <v>0.99692224665834439</v>
       </c>
       <c r="AP11">
-        <v>45.545153808519316</v>
+        <v>56.425477930352955</v>
       </c>
       <c r="AR11" t="s">
         <v>237</v>
@@ -7093,10 +7093,10 @@
         <v>416</v>
       </c>
       <c r="BC11">
-        <v>0.99402092584318991</v>
+        <v>0.99053075643264799</v>
       </c>
       <c r="BD11">
-        <v>109.61635954151812</v>
+        <v>173.60279873478748</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -7161,16 +7161,16 @@
         <v>242</v>
       </c>
       <c r="Y12" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="Z12" t="s">
         <v>275</v>
       </c>
       <c r="AA12">
-        <v>0.9981722170039925</v>
+        <v>0.99568371668484024</v>
       </c>
       <c r="AB12">
-        <v>33.509354926805031</v>
+        <v>79.131860777928608</v>
       </c>
       <c r="AD12" t="s">
         <v>237</v>
@@ -7200,13 +7200,13 @@
         <v>322</v>
       </c>
       <c r="AN12" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="AO12">
-        <v>0.99595483459575906</v>
+        <v>0.99725701149052537</v>
       </c>
       <c r="AP12">
-        <v>74.161365744417125</v>
+        <v>50.288122673700855</v>
       </c>
       <c r="AR12" t="s">
         <v>237</v>
@@ -7239,10 +7239,10 @@
         <v>418</v>
       </c>
       <c r="BC12">
-        <v>0.97533397850909798</v>
+        <v>0.98039565814133589</v>
       </c>
       <c r="BD12">
-        <v>452.21039399987052</v>
+        <v>359.41293407550836</v>
       </c>
     </row>
     <row r="13" spans="2:56">
@@ -7307,16 +7307,16 @@
         <v>244</v>
       </c>
       <c r="Y13" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="Z13" t="s">
         <v>276</v>
       </c>
       <c r="AA13">
-        <v>0.9958319028842455</v>
+        <v>0.99673728461460676</v>
       </c>
       <c r="AB13">
-        <v>76.415113788833068</v>
+        <v>59.816448732209111</v>
       </c>
       <c r="AD13" t="s">
         <v>237</v>
@@ -7343,16 +7343,16 @@
         <v>294</v>
       </c>
       <c r="AM13" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AN13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AO13">
-        <v>0.99857516825685033</v>
+        <v>0.99807547980555666</v>
       </c>
       <c r="AP13">
-        <v>26.121915291078167</v>
+        <v>35.282870231460656</v>
       </c>
       <c r="AR13" t="s">
         <v>237</v>
@@ -7453,16 +7453,16 @@
         <v>246</v>
       </c>
       <c r="Y14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Z14" t="s">
         <v>277</v>
       </c>
       <c r="AA14">
-        <v>0.9986195737404916</v>
+        <v>0.99709164861435029</v>
       </c>
       <c r="AB14">
-        <v>25.307814757654675</v>
+        <v>53.319775403577559</v>
       </c>
       <c r="AD14" t="s">
         <v>237</v>
@@ -7489,16 +7489,16 @@
         <v>296</v>
       </c>
       <c r="AM14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="AN14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="AO14">
-        <v>0.99624198670989172</v>
+        <v>0.99665105279570931</v>
       </c>
       <c r="AP14">
-        <v>68.896910318651507</v>
+        <v>61.397365411996212</v>
       </c>
       <c r="AR14" t="s">
         <v>237</v>
@@ -7528,7 +7528,7 @@
         <v>421</v>
       </c>
       <c r="BB14" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="BC14">
         <v>0.98183461816751461</v>
@@ -7599,16 +7599,16 @@
         <v>248</v>
       </c>
       <c r="Y15" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="Z15" t="s">
         <v>278</v>
       </c>
       <c r="AA15">
-        <v>0.99164479201276912</v>
+        <v>0.99541580702824473</v>
       </c>
       <c r="AB15">
-        <v>153.17881309923388</v>
+        <v>84.0435378155141</v>
       </c>
       <c r="AD15" t="s">
         <v>237</v>
@@ -7635,16 +7635,16 @@
         <v>298</v>
       </c>
       <c r="AM15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AN15" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="AO15">
-        <v>0.99665105279570931</v>
+        <v>0.99590345602074126</v>
       </c>
       <c r="AP15">
-        <v>61.397365411996212</v>
+        <v>75.103306286410302</v>
       </c>
       <c r="AR15" t="s">
         <v>237</v>
@@ -7745,16 +7745,16 @@
         <v>250</v>
       </c>
       <c r="Y16" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="Z16" t="s">
         <v>279</v>
       </c>
       <c r="AA16">
-        <v>0.99552574319771747</v>
+        <v>0.9981722170039925</v>
       </c>
       <c r="AB16">
-        <v>82.028041375179441</v>
+        <v>33.509354926805031</v>
       </c>
       <c r="AD16" t="s">
         <v>237</v>
@@ -7781,16 +7781,16 @@
         <v>300</v>
       </c>
       <c r="AM16" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AN16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AO16">
-        <v>0.99761292756299069</v>
+        <v>0.99446613913875159</v>
       </c>
       <c r="AP16">
-        <v>43.762994678503716</v>
+        <v>101.45411578955439</v>
       </c>
       <c r="AR16" t="s">
         <v>237</v>
@@ -7823,10 +7823,10 @@
         <v>425</v>
       </c>
       <c r="BC16">
-        <v>0.9878288138539939</v>
+        <v>0.98596601099553871</v>
       </c>
       <c r="BD16">
-        <v>223.13841267677765</v>
+        <v>257.2897984151241</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -7891,16 +7891,16 @@
         <v>252</v>
       </c>
       <c r="Y17" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="Z17" t="s">
         <v>280</v>
       </c>
       <c r="AA17">
-        <v>0.99856414548474748</v>
+        <v>0.99164479201276912</v>
       </c>
       <c r="AB17">
-        <v>26.323999446296273</v>
+        <v>153.17881309923388</v>
       </c>
       <c r="AD17" t="s">
         <v>237</v>
@@ -7927,16 +7927,16 @@
         <v>302</v>
       </c>
       <c r="AM17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AN17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AO17">
-        <v>0.99590345602074126</v>
+        <v>0.99821201020674788</v>
       </c>
       <c r="AP17">
-        <v>75.103306286410302</v>
+        <v>32.77981287628851</v>
       </c>
       <c r="AR17" t="s">
         <v>237</v>
@@ -7969,10 +7969,10 @@
         <v>427</v>
       </c>
       <c r="BC17">
-        <v>0.99503867375582744</v>
+        <v>0.992142345264865</v>
       </c>
       <c r="BD17">
-        <v>90.957647809829638</v>
+        <v>144.05700347747464</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -8037,16 +8037,16 @@
         <v>254</v>
       </c>
       <c r="Y18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="Z18" t="s">
         <v>281</v>
       </c>
       <c r="AA18">
-        <v>0.99837169372341228</v>
+        <v>0.99656426482871763</v>
       </c>
       <c r="AB18">
-        <v>29.852281737441412</v>
+        <v>62.988478140176163</v>
       </c>
       <c r="AD18" t="s">
         <v>237</v>
@@ -8073,16 +8073,16 @@
         <v>304</v>
       </c>
       <c r="AM18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AN18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AO18">
-        <v>0.99807547980555666</v>
+        <v>0.99562511313409086</v>
       </c>
       <c r="AP18">
-        <v>35.282870231460656</v>
+        <v>80.206259208334231</v>
       </c>
       <c r="AR18" t="s">
         <v>237</v>
@@ -8115,10 +8115,10 @@
         <v>429</v>
       </c>
       <c r="BC18">
-        <v>0.9960370911532308</v>
+        <v>0.99199988291996133</v>
       </c>
       <c r="BD18">
-        <v>72.653328857434573</v>
+        <v>146.66881313404267</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -8183,16 +8183,16 @@
         <v>256</v>
       </c>
       <c r="Y19" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="Z19" t="s">
         <v>282</v>
       </c>
       <c r="AA19">
-        <v>0.99781284363204548</v>
+        <v>0.9982917156958806</v>
       </c>
       <c r="AB19">
-        <v>40.097866745833329</v>
+        <v>31.318545575522229</v>
       </c>
       <c r="AD19" t="s">
         <v>237</v>
@@ -8219,16 +8219,16 @@
         <v>306</v>
       </c>
       <c r="AM19" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AN19" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="AO19">
-        <v>0.99239099026325794</v>
+        <v>0.9975157188831717</v>
       </c>
       <c r="AP19">
-        <v>139.49851184027145</v>
+        <v>45.545153808519316</v>
       </c>
       <c r="AR19" t="s">
         <v>237</v>
@@ -8261,10 +8261,10 @@
         <v>431</v>
       </c>
       <c r="BC19">
-        <v>0.98596601099553871</v>
+        <v>0.98560960960201449</v>
       </c>
       <c r="BD19">
-        <v>257.2897984151241</v>
+        <v>263.82382396306684</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -8329,16 +8329,16 @@
         <v>258</v>
       </c>
       <c r="Y20" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="Z20" t="s">
         <v>283</v>
       </c>
       <c r="AA20">
-        <v>0.99649838493007836</v>
+        <v>0.99781284363204548</v>
       </c>
       <c r="AB20">
-        <v>64.196276281897482</v>
+        <v>40.097866745833329</v>
       </c>
       <c r="AD20" t="s">
         <v>237</v>
@@ -8365,16 +8365,16 @@
         <v>308</v>
       </c>
       <c r="AM20" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AN20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AO20">
-        <v>0.99725701149052537</v>
+        <v>0.99826030196534266</v>
       </c>
       <c r="AP20">
-        <v>50.288122673700855</v>
+        <v>31.894463968718917</v>
       </c>
       <c r="AR20" t="s">
         <v>237</v>
@@ -8404,13 +8404,13 @@
         <v>432</v>
       </c>
       <c r="BB20" t="s">
-        <v>433</v>
+        <v>418</v>
       </c>
       <c r="BC20">
-        <v>0.992142345264865</v>
+        <v>0.9878288138539939</v>
       </c>
       <c r="BD20">
-        <v>144.05700347747464</v>
+        <v>223.13841267677765</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -8475,16 +8475,16 @@
         <v>260</v>
       </c>
       <c r="Y21" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="Z21" t="s">
         <v>284</v>
       </c>
       <c r="AA21">
-        <v>0.9982917156958806</v>
+        <v>0.99757939258365447</v>
       </c>
       <c r="AB21">
-        <v>31.318545575522229</v>
+        <v>44.377802633000776</v>
       </c>
       <c r="AD21" t="s">
         <v>237</v>
@@ -8511,16 +8511,16 @@
         <v>310</v>
       </c>
       <c r="AM21" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AN21" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AO21">
-        <v>0.99446613913875159</v>
+        <v>0.99761292756299069</v>
       </c>
       <c r="AP21">
-        <v>101.45411578955439</v>
+        <v>43.762994678503716</v>
       </c>
       <c r="AR21" t="s">
         <v>237</v>
@@ -8547,16 +8547,16 @@
         <v>369</v>
       </c>
       <c r="BA21" t="s">
+        <v>433</v>
+      </c>
+      <c r="BB21" t="s">
         <v>434</v>
       </c>
-      <c r="BB21" t="s">
-        <v>435</v>
-      </c>
       <c r="BC21">
-        <v>0.99199988291996133</v>
+        <v>0.97533397850909798</v>
       </c>
       <c r="BD21">
-        <v>146.66881313404267</v>
+        <v>452.21039399987052</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -8621,16 +8621,16 @@
         <v>262</v>
       </c>
       <c r="Y22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Z22" t="s">
         <v>285</v>
       </c>
       <c r="AA22">
-        <v>0.99757939258365447</v>
+        <v>0.99552574319771747</v>
       </c>
       <c r="AB22">
-        <v>44.377802633000776</v>
+        <v>82.028041375179441</v>
       </c>
       <c r="AD22" t="s">
         <v>237</v>
@@ -8657,16 +8657,16 @@
         <v>312</v>
       </c>
       <c r="AM22" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AN22" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AO22">
-        <v>0.99821201020674788</v>
+        <v>0.99239099026325794</v>
       </c>
       <c r="AP22">
-        <v>32.77981287628851</v>
+        <v>139.49851184027145</v>
       </c>
       <c r="AR22" t="s">
         <v>237</v>
@@ -8693,16 +8693,16 @@
         <v>371</v>
       </c>
       <c r="BA22" t="s">
+        <v>435</v>
+      </c>
+      <c r="BB22" t="s">
         <v>436</v>
       </c>
-      <c r="BB22" t="s">
-        <v>437</v>
-      </c>
       <c r="BC22">
-        <v>0.98560960960201449</v>
+        <v>0.99048115912556611</v>
       </c>
       <c r="BD22">
-        <v>263.82382396306684</v>
+        <v>174.51208269795416</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -8767,16 +8767,16 @@
         <v>264</v>
       </c>
       <c r="Y23" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="Z23" t="s">
         <v>286</v>
       </c>
       <c r="AA23">
-        <v>0.99568371668484024</v>
+        <v>0.99856414548474748</v>
       </c>
       <c r="AB23">
-        <v>79.131860777928608</v>
+        <v>26.323999446296273</v>
       </c>
       <c r="AD23" t="s">
         <v>237</v>
@@ -8803,16 +8803,16 @@
         <v>314</v>
       </c>
       <c r="AM23" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AN23" t="s">
-        <v>344</v>
+        <v>274</v>
       </c>
       <c r="AO23">
-        <v>0.99562511313409086</v>
+        <v>0.99595483459575906</v>
       </c>
       <c r="AP23">
-        <v>80.206259208334231</v>
+        <v>74.161365744417125</v>
       </c>
       <c r="AR23" t="s">
         <v>237</v>
@@ -8839,16 +8839,16 @@
         <v>373</v>
       </c>
       <c r="BA23" t="s">
+        <v>437</v>
+      </c>
+      <c r="BB23" t="s">
         <v>438</v>
       </c>
-      <c r="BB23" t="s">
-        <v>439</v>
-      </c>
       <c r="BC23">
-        <v>0.99342656473398216</v>
+        <v>0.99402264995370893</v>
       </c>
       <c r="BD23">
-        <v>120.51297987699346</v>
+        <v>109.58475084866993</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -8913,16 +8913,16 @@
         <v>266</v>
       </c>
       <c r="Y24" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="Z24" t="s">
         <v>287</v>
       </c>
       <c r="AA24">
-        <v>0.99673728461460676</v>
+        <v>0.99837169372341228</v>
       </c>
       <c r="AB24">
-        <v>59.816448732209111</v>
+        <v>29.852281737441412</v>
       </c>
       <c r="AD24" t="s">
         <v>237</v>
@@ -8955,10 +8955,10 @@
         <v>346</v>
       </c>
       <c r="AO24">
-        <v>0.99692224665834439</v>
+        <v>0.99857516825685033</v>
       </c>
       <c r="AP24">
-        <v>56.425477930352955</v>
+        <v>26.121915291078167</v>
       </c>
       <c r="AR24" t="s">
         <v>237</v>
@@ -8985,16 +8985,16 @@
         <v>375</v>
       </c>
       <c r="BA24" t="s">
+        <v>439</v>
+      </c>
+      <c r="BB24" t="s">
         <v>440</v>
       </c>
-      <c r="BB24" t="s">
-        <v>441</v>
-      </c>
       <c r="BC24">
-        <v>0.99728827252195684</v>
+        <v>0.9877150845460122</v>
       </c>
       <c r="BD24">
-        <v>49.715003764125143</v>
+        <v>225.22344998977596</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -9059,16 +9059,16 @@
         <v>268</v>
       </c>
       <c r="Y25" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="Z25" t="s">
         <v>288</v>
       </c>
       <c r="AA25">
-        <v>0.99709164861435029</v>
+        <v>0.9958319028842455</v>
       </c>
       <c r="AB25">
-        <v>53.319775403577559</v>
+        <v>76.415113788833068</v>
       </c>
       <c r="AD25" t="s">
         <v>237</v>
@@ -9101,10 +9101,10 @@
         <v>348</v>
       </c>
       <c r="AO25">
-        <v>0.99826030196534266</v>
+        <v>0.99624198670989172</v>
       </c>
       <c r="AP25">
-        <v>31.894463968718917</v>
+        <v>68.896910318651507</v>
       </c>
       <c r="AR25" t="s">
         <v>237</v>
@@ -9131,16 +9131,16 @@
         <v>377</v>
       </c>
       <c r="BA25" t="s">
+        <v>441</v>
+      </c>
+      <c r="BB25" t="s">
         <v>442</v>
       </c>
-      <c r="BB25" t="s">
-        <v>443</v>
-      </c>
       <c r="BC25">
-        <v>0.94957327345368925</v>
+        <v>0.96374055461874508</v>
       </c>
       <c r="BD25">
-        <v>924.48998668236334</v>
+        <v>664.7564986563408</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -9205,16 +9205,16 @@
         <v>270</v>
       </c>
       <c r="Y26" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="Z26" t="s">
         <v>289</v>
       </c>
       <c r="AA26">
-        <v>0.99656426482871763</v>
+        <v>0.9986195737404916</v>
       </c>
       <c r="AB26">
-        <v>62.988478140176163</v>
+        <v>25.307814757654675</v>
       </c>
       <c r="AR26" t="s">
         <v>237</v>
@@ -9241,16 +9241,16 @@
         <v>379</v>
       </c>
       <c r="BA26" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="BB26" t="s">
-        <v>445</v>
+        <v>275</v>
       </c>
       <c r="BC26">
-        <v>0.99048115912556611</v>
+        <v>0.98974923036021278</v>
       </c>
       <c r="BD26">
-        <v>174.51208269795416</v>
+        <v>187.93077672943278</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -9279,16 +9279,16 @@
         <v>381</v>
       </c>
       <c r="BA27" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="BB27" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="BC27">
-        <v>0.9955021345306051</v>
+        <v>0.99579892549254256</v>
       </c>
       <c r="BD27">
-        <v>82.460866938907401</v>
+        <v>77.019699303385977</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -9317,16 +9317,16 @@
         <v>383</v>
       </c>
       <c r="BA28" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="BB28" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="BC28">
-        <v>0.99514843803074871</v>
+        <v>0.99338832047077197</v>
       </c>
       <c r="BD28">
-        <v>88.945302769606073</v>
+        <v>121.21412470251306</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -9355,16 +9355,16 @@
         <v>385</v>
       </c>
       <c r="BA29" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="BB29" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="BC29">
-        <v>0.99052756852009682</v>
+        <v>0.99342656473398216</v>
       </c>
       <c r="BD29">
-        <v>173.66124379822571</v>
+        <v>120.51297987699346</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -9393,16 +9393,16 @@
         <v>387</v>
       </c>
       <c r="BA30" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="BB30" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="BC30">
-        <v>0.95113733831453195</v>
+        <v>0.99728827252195684</v>
       </c>
       <c r="BD30">
-        <v>895.81546423358179</v>
+        <v>49.715003764125143</v>
       </c>
     </row>
     <row r="31" spans="2:56">
@@ -9431,16 +9431,16 @@
         <v>389</v>
       </c>
       <c r="BA31" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="BB31" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="BC31">
-        <v>0.99402264995370893</v>
+        <v>0.94957327345368925</v>
       </c>
       <c r="BD31">
-        <v>109.58475084866993</v>
+        <v>924.48998668236334</v>
       </c>
     </row>
     <row r="32" spans="2:56">
@@ -9469,16 +9469,16 @@
         <v>391</v>
       </c>
       <c r="BA32" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="BB32" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="BC32">
-        <v>0.96374055461874508</v>
+        <v>0.99402092584318991</v>
       </c>
       <c r="BD32">
-        <v>664.7564986563408</v>
+        <v>109.61635954151812</v>
       </c>
     </row>
     <row r="33" spans="44:56">
@@ -9507,16 +9507,16 @@
         <v>393</v>
       </c>
       <c r="BA33" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="BB33" t="s">
-        <v>286</v>
+        <v>457</v>
       </c>
       <c r="BC33">
-        <v>0.98974923036021278</v>
+        <v>0.99503867375582744</v>
       </c>
       <c r="BD33">
-        <v>187.93077672943278</v>
+        <v>90.957647809829638</v>
       </c>
     </row>
     <row r="34" spans="44:56">
@@ -9545,16 +9545,16 @@
         <v>395</v>
       </c>
       <c r="BA34" t="s">
+        <v>458</v>
+      </c>
+      <c r="BB34" t="s">
         <v>459</v>
       </c>
-      <c r="BB34" t="s">
-        <v>460</v>
-      </c>
       <c r="BC34">
-        <v>0.99579892549254256</v>
+        <v>0.9960370911532308</v>
       </c>
       <c r="BD34">
-        <v>77.019699303385977</v>
+        <v>72.653328857434573</v>
       </c>
     </row>
     <row r="35" spans="44:56">
@@ -9583,16 +9583,16 @@
         <v>397</v>
       </c>
       <c r="BA35" t="s">
+        <v>460</v>
+      </c>
+      <c r="BB35" t="s">
         <v>461</v>
       </c>
-      <c r="BB35" t="s">
-        <v>453</v>
-      </c>
       <c r="BC35">
-        <v>0.99338832047077197</v>
+        <v>0.98395883577792953</v>
       </c>
       <c r="BD35">
-        <v>121.21412470251306</v>
+        <v>294.08801073795939</v>
       </c>
     </row>
     <row r="36" spans="44:56">
@@ -9627,10 +9627,10 @@
         <v>463</v>
       </c>
       <c r="BC36">
-        <v>0.96365973275398331</v>
+        <v>0.99439449087123744</v>
       </c>
       <c r="BD36">
-        <v>666.23823284363971</v>
+        <v>102.76766736064755</v>
       </c>
     </row>
     <row r="37" spans="44:56">
@@ -9665,10 +9665,10 @@
         <v>465</v>
       </c>
       <c r="BC37">
-        <v>0.99508487560623826</v>
+        <v>0.9955021345306051</v>
       </c>
       <c r="BD37">
-        <v>90.110613885632716</v>
+        <v>82.460866938907401</v>
       </c>
     </row>
     <row r="38" spans="44:56">
@@ -9703,10 +9703,10 @@
         <v>467</v>
       </c>
       <c r="BC38">
-        <v>0.9871879084242271</v>
+        <v>0.99514843803074871</v>
       </c>
       <c r="BD38">
-        <v>234.88834555583597</v>
+        <v>88.945302769606073</v>
       </c>
     </row>
     <row r="39" spans="44:56">
@@ -9741,10 +9741,10 @@
         <v>469</v>
       </c>
       <c r="BC39">
-        <v>0.98395883577792953</v>
+        <v>0.99052756852009682</v>
       </c>
       <c r="BD39">
-        <v>294.08801073795939</v>
+        <v>173.66124379822571</v>
       </c>
     </row>
     <row r="40" spans="44:56">
@@ -9776,13 +9776,13 @@
         <v>470</v>
       </c>
       <c r="BB40" t="s">
-        <v>471</v>
+        <v>447</v>
       </c>
       <c r="BC40">
-        <v>0.99439449087123744</v>
+        <v>0.95113733831453195</v>
       </c>
       <c r="BD40">
-        <v>102.76766736064755</v>
+        <v>895.81546423358179</v>
       </c>
     </row>
     <row r="41" spans="44:56">
@@ -9811,16 +9811,16 @@
         <v>409</v>
       </c>
       <c r="BA41" t="s">
+        <v>471</v>
+      </c>
+      <c r="BB41" t="s">
         <v>472</v>
       </c>
-      <c r="BB41" t="s">
-        <v>473</v>
-      </c>
       <c r="BC41">
-        <v>0.99053075643264799</v>
+        <v>0.96365973275398331</v>
       </c>
       <c r="BD41">
-        <v>173.60279873478748</v>
+        <v>666.23823284363971</v>
       </c>
     </row>
     <row r="42" spans="44:56">
@@ -9849,16 +9849,16 @@
         <v>411</v>
       </c>
       <c r="BA42" t="s">
+        <v>473</v>
+      </c>
+      <c r="BB42" t="s">
         <v>474</v>
       </c>
-      <c r="BB42" t="s">
-        <v>425</v>
-      </c>
       <c r="BC42">
-        <v>0.98039565814133589</v>
+        <v>0.99508487560623826</v>
       </c>
       <c r="BD42">
-        <v>359.41293407550836</v>
+        <v>90.110613885632716</v>
       </c>
     </row>
     <row r="43" spans="44:56">
@@ -9893,10 +9893,10 @@
         <v>476</v>
       </c>
       <c r="BC43">
-        <v>0.9877150845460122</v>
+        <v>0.9871879084242271</v>
       </c>
       <c r="BD43">
-        <v>225.22344998977596</v>
+        <v>234.88834555583597</v>
       </c>
     </row>
   </sheetData>
@@ -9905,7 +9905,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D0FA5E4-FEB2-4568-953C-8C71975D872C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E962DB0-E706-486A-83AC-B9BB9D5CA035}">
   <dimension ref="B9:Z43"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10017,7 +10017,7 @@
         <v>477</v>
       </c>
       <c r="K11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="L11">
         <v>8.3728062197205944</v>
@@ -10050,7 +10050,7 @@
         <v>507</v>
       </c>
       <c r="X11" t="s">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="Y11">
         <v>2.177</v>
@@ -10085,7 +10085,7 @@
         <v>479</v>
       </c>
       <c r="K12" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="L12">
         <v>42.531235680568031</v>
@@ -10118,7 +10118,7 @@
         <v>509</v>
       </c>
       <c r="X12" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="Y12">
         <v>32.750999999999998</v>
@@ -10153,7 +10153,7 @@
         <v>481</v>
       </c>
       <c r="K13" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="L13">
         <v>30.271312154499352</v>
@@ -10221,7 +10221,7 @@
         <v>483</v>
       </c>
       <c r="K14" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="L14">
         <v>22.688073076145226</v>
@@ -10254,7 +10254,7 @@
         <v>513</v>
       </c>
       <c r="X14" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="Y14">
         <v>30.484999999999999</v>
@@ -10289,7 +10289,7 @@
         <v>485</v>
       </c>
       <c r="K15" t="s">
-        <v>322</v>
+        <v>344</v>
       </c>
       <c r="L15">
         <v>29.120153762247021</v>
@@ -10322,7 +10322,7 @@
         <v>515</v>
       </c>
       <c r="X15" t="s">
-        <v>428</v>
+        <v>458</v>
       </c>
       <c r="Y15">
         <v>6.726</v>
@@ -10357,7 +10357,7 @@
         <v>487</v>
       </c>
       <c r="K16" t="s">
-        <v>323</v>
+        <v>345</v>
       </c>
       <c r="L16">
         <v>10.867385180190169</v>
@@ -10390,7 +10390,7 @@
         <v>517</v>
       </c>
       <c r="X16" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="Y16">
         <v>33.183</v>
@@ -10425,7 +10425,7 @@
         <v>489</v>
       </c>
       <c r="K17" t="s">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="L17">
         <v>32.115075062865692</v>
@@ -10458,7 +10458,7 @@
         <v>519</v>
       </c>
       <c r="X17" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="Y17">
         <v>3.617</v>
@@ -10493,7 +10493,7 @@
         <v>491</v>
       </c>
       <c r="K18" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="L18">
         <v>9.0868240253443027</v>
@@ -10561,7 +10561,7 @@
         <v>493</v>
       </c>
       <c r="K19" t="s">
-        <v>320</v>
+        <v>336</v>
       </c>
       <c r="L19">
         <v>18.016423245563796</v>
@@ -10594,7 +10594,7 @@
         <v>523</v>
       </c>
       <c r="X19" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="Y19">
         <v>60.06</v>
@@ -10629,7 +10629,7 @@
         <v>495</v>
       </c>
       <c r="K20" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="L20">
         <v>0.75250112047637663</v>
@@ -10662,7 +10662,7 @@
         <v>525</v>
       </c>
       <c r="X20" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="Y20">
         <v>70.188999999999993</v>
@@ -10697,7 +10697,7 @@
         <v>497</v>
       </c>
       <c r="K21" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="L21">
         <v>18.381813037942475</v>
@@ -10730,7 +10730,7 @@
         <v>527</v>
       </c>
       <c r="X21" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="Y21">
         <v>40.698999999999998</v>
@@ -10765,7 +10765,7 @@
         <v>499</v>
       </c>
       <c r="K22" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="L22">
         <v>4.5221914845937041</v>
@@ -10798,7 +10798,7 @@
         <v>529</v>
       </c>
       <c r="X22" t="s">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="Y22">
         <v>28.895</v>
@@ -10833,7 +10833,7 @@
         <v>501</v>
       </c>
       <c r="K23" t="s">
-        <v>325</v>
+        <v>347</v>
       </c>
       <c r="L23">
         <v>8.2953562793919264</v>
@@ -10866,7 +10866,7 @@
         <v>531</v>
       </c>
       <c r="X23" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="Y23">
         <v>259.62099999999998</v>
@@ -10901,7 +10901,7 @@
         <v>503</v>
       </c>
       <c r="K24" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="L24">
         <v>1.2792726734837132</v>
@@ -10934,7 +10934,7 @@
         <v>533</v>
       </c>
       <c r="X24" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="Y24">
         <v>96.406999999999996</v>
@@ -10969,7 +10969,7 @@
         <v>505</v>
       </c>
       <c r="K25" t="s">
-        <v>345</v>
+        <v>320</v>
       </c>
       <c r="L25">
         <v>1.6182682752282065</v>
@@ -11002,7 +11002,7 @@
         <v>535</v>
       </c>
       <c r="X25" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="Y25">
         <v>218.93100000000001</v>
@@ -11037,7 +11037,7 @@
         <v>537</v>
       </c>
       <c r="X26" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="Y26">
         <v>164.86799999999999</v>
@@ -11072,7 +11072,7 @@
         <v>539</v>
       </c>
       <c r="X27" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="Y27">
         <v>177.54</v>
@@ -11107,7 +11107,7 @@
         <v>541</v>
       </c>
       <c r="X28" t="s">
-        <v>426</v>
+        <v>456</v>
       </c>
       <c r="Y28">
         <v>32.006</v>
@@ -11142,7 +11142,7 @@
         <v>543</v>
       </c>
       <c r="X29" t="s">
-        <v>472</v>
+        <v>415</v>
       </c>
       <c r="Y29">
         <v>92.117999999999995</v>
@@ -11212,7 +11212,7 @@
         <v>547</v>
       </c>
       <c r="X31" t="s">
-        <v>444</v>
+        <v>435</v>
       </c>
       <c r="Y31">
         <v>55.912999999999997</v>
@@ -11247,7 +11247,7 @@
         <v>549</v>
       </c>
       <c r="X32" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="Y32">
         <v>45.517000000000003</v>
@@ -11282,7 +11282,7 @@
         <v>551</v>
       </c>
       <c r="X33" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="Y33">
         <v>76.210999999999999</v>
@@ -11317,7 +11317,7 @@
         <v>553</v>
       </c>
       <c r="X34" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="Y34">
         <v>44.996000000000002</v>
@@ -11352,7 +11352,7 @@
         <v>555</v>
       </c>
       <c r="X35" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="Y35">
         <v>69.513999999999996</v>
@@ -11387,7 +11387,7 @@
         <v>557</v>
       </c>
       <c r="X36" t="s">
-        <v>415</v>
+        <v>454</v>
       </c>
       <c r="Y36">
         <v>60.743000000000002</v>
@@ -11422,7 +11422,7 @@
         <v>559</v>
       </c>
       <c r="X37" t="s">
-        <v>474</v>
+        <v>417</v>
       </c>
       <c r="Y37">
         <v>72.956000000000003</v>
@@ -11457,7 +11457,7 @@
         <v>561</v>
       </c>
       <c r="X38" t="s">
-        <v>458</v>
+        <v>443</v>
       </c>
       <c r="Y38">
         <v>19.841000000000001</v>
@@ -11492,7 +11492,7 @@
         <v>563</v>
       </c>
       <c r="X39" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="Y39">
         <v>138.42500000000001</v>
@@ -11527,7 +11527,7 @@
         <v>565</v>
       </c>
       <c r="X40" t="s">
-        <v>475</v>
+        <v>439</v>
       </c>
       <c r="Y40">
         <v>142.483</v>
@@ -11562,7 +11562,7 @@
         <v>567</v>
       </c>
       <c r="X41" t="s">
-        <v>454</v>
+        <v>437</v>
       </c>
       <c r="Y41">
         <v>20.327999999999999</v>
@@ -11597,7 +11597,7 @@
         <v>569</v>
       </c>
       <c r="X42" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="Y42">
         <v>65.320999999999998</v>
@@ -11632,7 +11632,7 @@
         <v>571</v>
       </c>
       <c r="X43" t="s">
-        <v>459</v>
+        <v>444</v>
       </c>
       <c r="Y43">
         <v>32.902000000000001</v>
@@ -11647,7 +11647,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C167C9A6-CF52-4DA2-8528-B84871055501}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB7543C-A9AC-463B-A3D3-9B62CD70D42F}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>